<commit_message>
rfactor by creating an independent session recorder
</commit_message>
<xml_diff>
--- a/tools/GANTT/Cool_Spine_GANTT.xlsx
+++ b/tools/GANTT/Cool_Spine_GANTT.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cool_Spine_Roadmap_October_2026" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cool_Spine_Roadmap_October_2026'!$A$5:$AW$110</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cool_Spine_Roadmap_October_2026'!$A$5:$AW$154</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="mmm\ yyyy"/>
     <numFmt numFmtId="165" formatCode="dd\-mmm\-yy"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -48,8 +48,14 @@
       <color theme="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -73,6 +79,12 @@
         <fgColor theme="6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="13">
     <border>
@@ -226,7 +238,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -269,20 +281,40 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFF2CC"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -680,20 +712,24 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr filterMode="1">
+  <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AW110"/>
+  <dimension ref="A1:AW154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="72.7265625" customWidth="1" style="26" min="1" max="1"/>
-    <col width="30.7265625" customWidth="1" style="16" min="2" max="2"/>
+    <col width="65.6328125" customWidth="1" style="36" min="1" max="1"/>
+    <col width="17.1796875" customWidth="1" style="16" min="2" max="2"/>
     <col width="9.1796875" customWidth="1" style="10" min="3" max="3"/>
-    <col width="9.1796875" customWidth="1" style="26" min="4" max="22"/>
-    <col width="9.1796875" customWidth="1" style="27" min="23" max="23"/>
-    <col width="9.1796875" customWidth="1" style="26" min="38" max="38"/>
-    <col width="9.36328125" bestFit="1" customWidth="1" style="26" min="39" max="39"/>
+    <col width="9.1796875" customWidth="1" style="36" min="4" max="22"/>
+    <col width="9.1796875" customWidth="1" style="33" min="23" max="23"/>
+    <col width="9.08984375" bestFit="1" customWidth="1" style="36" min="24" max="24"/>
+    <col width="9.1796875" bestFit="1" customWidth="1" style="36" min="25" max="26"/>
+    <col width="9.36328125" bestFit="1" customWidth="1" style="36" min="27" max="29"/>
+    <col width="9.1796875" bestFit="1" customWidth="1" style="36" min="35" max="35"/>
+    <col width="9.1796875" customWidth="1" style="36" min="38" max="38"/>
+    <col width="9.36328125" bestFit="1" customWidth="1" style="36" min="39" max="39"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -726,17 +762,17 @@
           <t>Q3 2026</t>
         </is>
       </c>
-      <c r="W2" s="28" t="inlineStr">
+      <c r="W2" s="34" t="inlineStr">
         <is>
           <t>Q4 2026</t>
         </is>
       </c>
-      <c r="X2" s="29" t="n"/>
-      <c r="Y2" s="29" t="n"/>
-      <c r="Z2" s="29" t="n"/>
-      <c r="AA2" s="29" t="n"/>
-      <c r="AB2" s="29" t="n"/>
-      <c r="AC2" s="28" t="n"/>
+      <c r="X2" s="35" t="n"/>
+      <c r="Y2" s="35" t="n"/>
+      <c r="Z2" s="35" t="n"/>
+      <c r="AA2" s="35" t="n"/>
+      <c r="AB2" s="35" t="n"/>
+      <c r="AC2" s="34" t="n"/>
       <c r="AD2" t="inlineStr">
         <is>
           <t>Q1 2027</t>
@@ -758,7 +794,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1" s="26" thickBot="1">
+    <row r="3" ht="15.75" customHeight="1" s="36" thickBot="1">
       <c r="C3" s="18" t="n">
         <v>46023</v>
       </c>
@@ -961,15 +997,15 @@
         </is>
       </c>
     </row>
-    <row r="6" hidden="1" s="26">
-      <c r="A6" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="37" t="inlineStr">
         <is>
           <t>Planning &amp; Preparation</t>
         </is>
       </c>
     </row>
-    <row r="7" hidden="1" s="26">
-      <c r="A7" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="37" t="inlineStr">
         <is>
           <t>Discussion with CoolSpine Team</t>
         </is>
@@ -980,16 +1016,16 @@
         </is>
       </c>
     </row>
-    <row r="8" hidden="1" s="26">
-      <c r="A8" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="37" t="inlineStr">
         <is>
           <t>Medical Device Design course project kickoff</t>
         </is>
       </c>
       <c r="C8" s="12" t="n"/>
     </row>
-    <row r="9" hidden="1" s="26">
-      <c r="A9" s="2" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="37" t="inlineStr">
         <is>
           <t>Team Established</t>
         </is>
@@ -1002,7 +1038,7 @@
       <c r="C9" s="12" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="37" t="inlineStr">
         <is>
           <t>Onsite with Sage PD – detailed project review and establishment of responsibilities</t>
         </is>
@@ -1014,16 +1050,16 @@
       </c>
       <c r="C10" s="12" t="n"/>
     </row>
-    <row r="11" hidden="1" s="26">
-      <c r="A11" s="2" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="37" t="inlineStr">
         <is>
           <t>Establishment of design Functional Requirements</t>
         </is>
       </c>
       <c r="D11" s="13" t="n"/>
     </row>
-    <row r="12" hidden="1" s="26">
-      <c r="A12" s="2" t="n"/>
+    <row r="12">
+      <c r="A12" s="37" t="n"/>
       <c r="D12" s="13" t="n"/>
     </row>
     <row r="13">
@@ -1034,189 +1070,189 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="37" t="inlineStr">
+        <is>
+          <t>Strategy Presentations</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>Studied refrigeration v. thermoelectric cooling</t>
+        </is>
+      </c>
+      <c r="E15" s="13" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="37" t="inlineStr">
+        <is>
+          <t>Reviewed Zoll system</t>
+        </is>
+      </c>
+      <c r="E16" s="13" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>Concept Presentation</t>
+        </is>
+      </c>
+      <c r="B17" s="16" t="inlineStr">
+        <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="D13" s="13" t="n"/>
-    </row>
-    <row r="14" hidden="1" s="26">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Strategy Presentations</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="n"/>
-    </row>
-    <row r="15" hidden="1" s="26">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Studied refrigeration v. thermoelectric cooling</t>
-        </is>
-      </c>
-      <c r="E15" s="13" t="n"/>
-    </row>
-    <row r="16" hidden="1" s="26">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Reviewed Zoll system</t>
-        </is>
-      </c>
-      <c r="E16" s="13" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Concept Presentation</t>
-        </is>
-      </c>
-      <c r="B17" s="16" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
       <c r="E17" s="13" t="n"/>
     </row>
-    <row r="18" hidden="1" s="26">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="37" t="inlineStr">
         <is>
           <t>De-selection of thermoelectric cooling</t>
         </is>
       </c>
       <c r="E18" s="13" t="n"/>
     </row>
-    <row r="19" hidden="1" s="26">
-      <c r="A19" s="2" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="37" t="inlineStr">
         <is>
           <t>Hub connector review with Sage</t>
         </is>
       </c>
       <c r="F19" s="13" t="n"/>
     </row>
-    <row r="20" hidden="1" s="26">
-      <c r="A20" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="37" t="inlineStr">
         <is>
           <t>Modelling of worst-case maximum cooling</t>
         </is>
       </c>
       <c r="F20" s="13" t="n"/>
     </row>
-    <row r="21" hidden="1" s="26">
-      <c r="A21" s="2" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="37" t="inlineStr">
         <is>
           <t>Fabrication and assembly of test fluid cooling loop</t>
         </is>
       </c>
       <c r="F21" s="13" t="n"/>
     </row>
-    <row r="22" hidden="1" s="26">
-      <c r="A22" s="2" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="37" t="inlineStr">
         <is>
           <t>Testing</t>
         </is>
       </c>
       <c r="F22" s="13" t="n"/>
     </row>
-    <row r="23" hidden="1" s="26">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="37" t="inlineStr">
         <is>
           <t>Preliminary UIUX, including pump controls and alarms</t>
         </is>
       </c>
       <c r="G23" s="13" t="n"/>
     </row>
-    <row r="24" hidden="1" s="26">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="37" t="inlineStr">
         <is>
           <t>Full system concept design established</t>
         </is>
       </c>
       <c r="G24" s="13" t="n"/>
     </row>
-    <row r="25" hidden="1" s="26">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="37" t="inlineStr">
         <is>
           <t>Model of required cooling power and cooling power v time</t>
         </is>
       </c>
       <c r="G25" s="13" t="n"/>
     </row>
-    <row r="26" hidden="1" s="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="37" t="inlineStr">
         <is>
           <t>Bench testing</t>
         </is>
       </c>
       <c r="G26" s="13" t="n"/>
     </row>
-    <row r="27" hidden="1" s="26">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="37" t="inlineStr">
         <is>
           <t>Course 2.75 - Final presentations</t>
         </is>
       </c>
       <c r="G27" s="13" t="n"/>
     </row>
-    <row r="28" hidden="1" s="26"/>
-    <row r="29" hidden="1" s="26">
-      <c r="A29" s="2" t="inlineStr">
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="37" t="inlineStr">
         <is>
           <t>Thermistor selection &amp; meeting with Sage and Amphenol</t>
         </is>
       </c>
       <c r="H29" s="13" t="n"/>
     </row>
-    <row r="30" hidden="1" s="26">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="37" t="inlineStr">
         <is>
           <t>Assembly of pressure and temperature sensing modules</t>
         </is>
       </c>
       <c r="H30" s="13" t="n"/>
     </row>
-    <row r="31" hidden="1" s="26">
-      <c r="A31" s="2" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="37" t="inlineStr">
         <is>
           <t>Finalization of UIUX</t>
         </is>
       </c>
       <c r="H31" s="13" t="n"/>
     </row>
-    <row r="32" hidden="1" s="26">
-      <c r="A32" s="2" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="37" t="inlineStr">
         <is>
           <t>Risk &amp; DMEA Review with Sage</t>
         </is>
       </c>
       <c r="I32" s="13" t="n"/>
     </row>
-    <row r="33" hidden="1" s="26">
-      <c r="A33" s="2" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="37" t="inlineStr">
         <is>
           <t>Onsite catheter testing at MIT with Sage</t>
         </is>
       </c>
       <c r="I33" s="13" t="n"/>
     </row>
-    <row r="34" hidden="1" s="26">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="37" t="inlineStr">
         <is>
           <t>Revision of cooling system design to support cartridge design</t>
         </is>
       </c>
       <c r="I34" s="13" t="n"/>
     </row>
-    <row r="35" hidden="1" s="26">
-      <c r="A35" s="2" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="37" t="inlineStr">
         <is>
           <t>Preliminary discussion with Aspen</t>
         </is>
       </c>
       <c r="I35" s="13" t="n"/>
     </row>
-    <row r="36" hidden="1" s="26">
-      <c r="A36" s="32" t="inlineStr">
-        <is>
-          <t>Check with Aspen (supplier) if the gas we are using may be used in the operating room, and if they have any experience with it in medical devices</t>
+    <row r="36">
+      <c r="A36" s="28" t="inlineStr">
+        <is>
+          <t>Propane R290, Check with Aspen (supplier) if the gas we are using may be used in the operating room, and if they have any experience with it in medical devices</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1224,10 +1260,10 @@
           <t>Current Sprint</t>
         </is>
       </c>
-      <c r="X36" s="31" t="n"/>
-    </row>
-    <row r="37" hidden="1" s="26">
-      <c r="A37" s="2" t="inlineStr">
+      <c r="X36" s="27" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="37" t="inlineStr">
         <is>
           <t>Catheter test to failure</t>
         </is>
@@ -1238,568 +1274,870 @@
       <c r="I38" s="13" t="n"/>
       <c r="X38" s="10" t="n"/>
     </row>
-    <row r="39" hidden="1" s="26">
-      <c r="A39" s="1" t="inlineStr">
+    <row r="39">
+      <c r="I39" s="13" t="n"/>
+    </row>
+    <row r="40">
+      <c r="I40" s="13" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr">
         <is>
           <t>Catheter power</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="C39" s="14" t="n"/>
-    </row>
-    <row r="40" hidden="1" s="26">
-      <c r="A40" s="5" t="inlineStr">
+      <c r="C41" s="14" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="38" t="inlineStr">
         <is>
           <t>Analytical Model creation - catheder to tissue (to be verified)</t>
         </is>
       </c>
-      <c r="C40" s="15" t="n"/>
-    </row>
-    <row r="41" hidden="1" s="26">
-      <c r="A41" s="5" t="inlineStr">
+      <c r="C42" s="15" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="38" t="inlineStr">
         <is>
           <t>Cathether design fixed (SAGE)</t>
         </is>
       </c>
-      <c r="C41" s="15" t="n"/>
-    </row>
-    <row r="42" hidden="1" s="26">
-      <c r="A42" s="5" t="inlineStr">
+      <c r="C43" s="15" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="38" t="inlineStr">
         <is>
           <t>Cool plates and cartrige design</t>
         </is>
       </c>
-      <c r="C42" s="15" t="n"/>
-    </row>
-    <row r="43" hidden="1" s="26">
-      <c r="A43" s="5" t="inlineStr">
+      <c r="C44" s="15" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="38" t="inlineStr">
         <is>
           <t>Banchmark catheder test (body phantom) 0C -&gt; 40W at y ml/min</t>
         </is>
       </c>
-      <c r="C43" s="15" t="n"/>
-    </row>
-    <row r="44" hidden="1" s="26">
-      <c r="A44" s="5" t="inlineStr">
+      <c r="C45" s="15" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="38" t="inlineStr">
+        <is>
+          <t>Termistors study</t>
+        </is>
+      </c>
+      <c r="X46" s="13" t="n"/>
+    </row>
+    <row r="47"/>
+    <row r="48"/>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="38" t="n"/>
+      <c r="C50" s="15" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="37" t="n"/>
+      <c r="C51" s="15" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>Cartrige</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+      <c r="C52" s="14" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="38" t="inlineStr">
+        <is>
+          <t>Analytical Model creation</t>
+        </is>
+      </c>
+      <c r="C53" s="14" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="38" t="inlineStr">
+        <is>
+          <t>Manufacture a 3d printed cartrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="38" t="inlineStr">
+        <is>
+          <t>Test in ice bath</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="38" t="inlineStr">
+        <is>
+          <t>Test with cool plate system ?</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="38" t="inlineStr">
+        <is>
+          <t>Cooling System</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="38" t="inlineStr">
         <is>
           <t>Current coldplate (-2-1) testing -&gt; -27W</t>
         </is>
       </c>
-      <c r="C44" s="15" t="n"/>
-    </row>
-    <row r="45" hidden="1" s="26">
-      <c r="A45" s="5" t="inlineStr">
+      <c r="C58" s="15" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="38" t="inlineStr">
         <is>
           <t>Tuning of the current system</t>
         </is>
       </c>
-      <c r="C45" s="15" t="n"/>
-    </row>
-    <row r="46" hidden="1" s="26">
-      <c r="A46" s="5" t="inlineStr">
+      <c r="C59" s="15" t="n"/>
+      <c r="X59" s="13" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="38" t="inlineStr">
         <is>
           <t>CONTINGENCY PLAN (if we need: bigger coldplate, 10weeks - 10K ?)</t>
         </is>
       </c>
-      <c r="C46" s="15" t="n"/>
-    </row>
-    <row r="47" hidden="1" s="26">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>CONTINGENCY 2</t>
-        </is>
-      </c>
-      <c r="C47" s="15" t="n"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n"/>
-      <c r="C48" s="15" t="n"/>
-    </row>
-    <row r="49" hidden="1" s="26">
-      <c r="A49" s="17" t="inlineStr">
-        <is>
-          <t>Cartrige</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
+      <c r="C60" s="15" t="n"/>
+      <c r="Y60" s="13" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="38" t="inlineStr">
+        <is>
+          <t>CONTINGENCY 2 (think about peltier ...)</t>
+        </is>
+      </c>
+      <c r="C61" s="15" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Oder second cartrige from "R&amp;D" </t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="n"/>
+      <c r="X62" s="13" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="38" t="inlineStr">
+        <is>
+          <t>Test the second cartrige</t>
+        </is>
+      </c>
+      <c r="C63" s="15" t="n"/>
+      <c r="Y63" s="13" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="38" t="n"/>
+      <c r="C64" s="15" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">V2 - including the deboubler ? </t>
+        </is>
+      </c>
+      <c r="C65" s="15" t="n"/>
+      <c r="Z65" s="13" t="n"/>
+      <c r="AA65" s="13" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="38" t="inlineStr">
+        <is>
+          <t>Manufacture final from material</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="38" t="n"/>
+      <c r="C67" s="15" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="17" t="inlineStr">
+        <is>
+          <t>Tubing</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
-      <c r="C49" s="14" t="n"/>
-    </row>
-    <row r="50" hidden="1" s="26">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>Analytical Model creation</t>
-        </is>
-      </c>
-      <c r="C50" s="14" t="n"/>
-    </row>
-    <row r="51" hidden="1" s="26">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>Manufacture a 3d printed cartrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" hidden="1" s="26">
-      <c r="A52" s="5" t="inlineStr">
-        <is>
-          <t>Test in ice bath</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" hidden="1" s="26">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>Test with cool plate system ?</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" hidden="1" s="26">
-      <c r="A54" s="5" t="inlineStr">
-        <is>
-          <t>Cooling System</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="n"/>
-    </row>
-    <row r="56" hidden="1" s="26">
-      <c r="A56" s="17" t="inlineStr">
-        <is>
-          <t>Tubing</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
+    </row>
+    <row r="69">
+      <c r="A69" s="38" t="inlineStr">
+        <is>
+          <t>Conduct test with the Tygoon PVC (10% drop at after 20min)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="25" t="inlineStr">
+        <is>
+          <t>Conduct tests for the current tubing, moving it along the length every 30min</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Current Sprint</t>
+        </is>
+      </c>
+      <c r="X70" s="27" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="38" t="inlineStr">
+        <is>
+          <t>Identify alternate tubing</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="38" t="inlineStr">
+        <is>
+          <t>Test &amp; Verify</t>
+        </is>
+      </c>
+      <c r="X72" s="13" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="38" t="inlineStr">
+        <is>
+          <t>masterflex qualified sesrs</t>
+        </is>
+      </c>
+      <c r="Y73" s="13" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3 materials: 6h approriate temp and flowrate, closed lines, </t>
+        </is>
+      </c>
+      <c r="Y74" s="13" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="38" t="inlineStr">
+        <is>
+          <t>reach out to 2 different tubing companies</t>
+        </is>
+      </c>
+      <c r="Y75" s="13" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="38" t="inlineStr">
+        <is>
+          <t>move charges venture well</t>
+        </is>
+      </c>
+      <c r="Z76" s="13" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="38" t="inlineStr">
+        <is>
+          <t>use silicon caulking</t>
+        </is>
+      </c>
+      <c r="Z77" s="13" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="38" t="inlineStr">
+        <is>
+          <t>create new sensors Tshaped connectors</t>
+        </is>
+      </c>
+      <c r="Y78" s="13" t="n"/>
+    </row>
+    <row r="79"/>
+    <row r="80">
+      <c r="A80" s="17" t="inlineStr">
+        <is>
+          <t>Housing  P1.5</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
     </row>
-    <row r="57" hidden="1" s="26">
-      <c r="A57" s="5" t="inlineStr">
-        <is>
-          <t>Conduct test with the Tygoon PVC (10% drop at after 20min)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" hidden="1" s="26">
-      <c r="A58" s="25" t="inlineStr">
-        <is>
-          <t>Conduct tests for the current tubing, moving it along the length every 30min</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
+    <row r="81">
+      <c r="A81" s="38" t="inlineStr">
+        <is>
+          <t>CAD modeling</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="38" t="inlineStr">
+        <is>
+          <t>Order</t>
+        </is>
+      </c>
+      <c r="V82" s="13" t="n"/>
+      <c r="W82" s="30" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="38" t="inlineStr">
+        <is>
+          <t>Build</t>
+        </is>
+      </c>
+      <c r="X83" s="13" t="n"/>
+      <c r="Y83" s="13" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="38" t="inlineStr">
+        <is>
+          <t>Assemble &amp; Verify</t>
+        </is>
+      </c>
+      <c r="Y84" s="13" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="37" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t>Probes</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="38" t="inlineStr">
+        <is>
+          <t>Evaluate probes from previous work --&gt; probes insufficient --&gt; new probes required</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="7" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="38" t="inlineStr">
+        <is>
+          <t>Manufacture</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="38" t="inlineStr">
+        <is>
+          <t>Test &amp; Integrate</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="25" t="inlineStr">
+        <is>
+          <t>Design new probes for the animal study</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
         <is>
           <t>Current Sprint</t>
         </is>
       </c>
-      <c r="X58" s="31" t="n"/>
-    </row>
-    <row r="59" hidden="1" s="26">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>Identify alternate tubing</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>Test &amp; Verify</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" hidden="1" s="26"/>
-    <row r="62" hidden="1" s="26">
-      <c r="A62" s="17" t="inlineStr">
-        <is>
-          <t>Housing  P1.5</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
+      <c r="X91" s="13" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="31" t="inlineStr">
+        <is>
+          <t>Order needls and extension cables</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Current Sprint</t>
+        </is>
+      </c>
+      <c r="X92" s="13" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="25" t="inlineStr">
+        <is>
+          <t>Integrate and test the probes</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Next Sprint</t>
+        </is>
+      </c>
+      <c r="Y93" s="13" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="31" t="inlineStr">
+        <is>
+          <t>WIRE THE Peristaltic pump limit switch</t>
+        </is>
+      </c>
+      <c r="Y94" s="13" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="37" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>Liquid level sensor</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="37" t="inlineStr">
+        <is>
+          <t>Try the sensro we allready have</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="37" t="inlineStr">
+        <is>
+          <t>Send a quote</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="37" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="37" t="inlineStr">
+        <is>
+          <t>Dboubler</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="37" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="37" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="17" t="inlineStr">
+        <is>
+          <t>Circut Board</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
     </row>
-    <row r="63" hidden="1" s="26">
-      <c r="A63" s="5" t="inlineStr">
-        <is>
-          <t>CAD modeling</t>
-        </is>
-      </c>
-    </row>
-    <row r="64" hidden="1" s="26">
-      <c r="A64" s="5" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="38" t="inlineStr">
+        <is>
+          <t>Design</t>
+        </is>
+      </c>
+      <c r="V104" s="13" t="n"/>
+      <c r="W104" s="30" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="38" t="inlineStr">
         <is>
           <t>Order</t>
         </is>
       </c>
-    </row>
-    <row r="65" hidden="1" s="26">
-      <c r="A65" s="5" t="inlineStr">
+      <c r="W105" s="30" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="38" t="inlineStr">
+        <is>
+          <t>Integrate &amp; Test</t>
+        </is>
+      </c>
+      <c r="X106" s="13" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="38" t="inlineStr">
+        <is>
+          <t>Revise</t>
+        </is>
+      </c>
+      <c r="Y107" s="13" t="n"/>
+      <c r="Z107" s="13" t="n"/>
+      <c r="AA107" s="13" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="38" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="17" t="inlineStr">
+        <is>
+          <t>Battery System</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="38" t="inlineStr">
+        <is>
+          <t>Integrate the Battery</t>
+        </is>
+      </c>
+      <c r="X110" s="13" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="38" t="inlineStr">
+        <is>
+          <t>Implement UI and Error cases</t>
+        </is>
+      </c>
+      <c r="X111" s="13" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="38" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="X112" s="13" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="38" t="inlineStr">
+        <is>
+          <t>Simulate 30min operation</t>
+        </is>
+      </c>
+      <c r="Y113" s="13" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="25" t="inlineStr">
+        <is>
+          <t>Test whether USB-C input is an option</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Current Sprint</t>
+        </is>
+      </c>
+      <c r="X114" s="27" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="25" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="37" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="17" t="inlineStr">
+        <is>
+          <t>Sage Test Setup</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Epic</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="38" t="inlineStr">
+        <is>
+          <t>Design and order</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="38" t="inlineStr">
         <is>
           <t>Build</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="5" t="inlineStr">
-        <is>
-          <t>Assemble &amp; Verify</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" hidden="1" s="26">
-      <c r="A67" s="2" t="n"/>
-    </row>
-    <row r="68" hidden="1" s="26">
-      <c r="A68" s="17" t="inlineStr">
-        <is>
-          <t>Probes</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
+    <row r="120"/>
+    <row r="121">
+      <c r="A121" s="17" t="inlineStr">
+        <is>
+          <t>Prep for Animal Study</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
     </row>
-    <row r="69" hidden="1" s="26">
-      <c r="A69" s="5" t="inlineStr">
-        <is>
-          <t>Evaluate probes from previous work --&gt; probes insufficient --&gt; new probes required</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" hidden="1" s="26">
-      <c r="A70" s="7" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="5" t="inlineStr">
-        <is>
-          <t>Manufacture</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" hidden="1" s="26">
-      <c r="A72" s="5" t="inlineStr">
-        <is>
-          <t>Test &amp; Integrate</t>
-        </is>
-      </c>
-    </row>
-    <row r="73" hidden="1" s="26">
-      <c r="A73" s="25" t="inlineStr">
-        <is>
-          <t>Design new probes for the animal study</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Current Sprint</t>
-        </is>
-      </c>
-      <c r="X73" s="13" t="n"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="25" t="inlineStr">
-        <is>
-          <t>Integrate and test the probes</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Next Sprint</t>
-        </is>
-      </c>
-      <c r="Y74" s="13" t="n"/>
-    </row>
-    <row r="75" hidden="1" s="26">
-      <c r="A75" s="2" t="n"/>
-    </row>
-    <row r="76" hidden="1" s="26">
-      <c r="A76" s="17" t="inlineStr">
-        <is>
-          <t>Circut Board</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="38" t="inlineStr">
+        <is>
+          <t>Study previous experiments</t>
+        </is>
+      </c>
+      <c r="W122" s="30" t="n"/>
+      <c r="X122" s="13" t="n"/>
+      <c r="Y122" s="13" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="38" t="inlineStr">
+        <is>
+          <t>Make contact with the Ohaio people</t>
+        </is>
+      </c>
+      <c r="X123" s="13" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="38" t="inlineStr">
+        <is>
+          <t>Desing the Study protocol - especially probe placement</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="38" t="inlineStr">
+        <is>
+          <t>Freeze the software/hardware version and conduct final verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="3" t="inlineStr">
+        <is>
+          <t>Software</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="37" t="inlineStr">
+        <is>
+          <t>Move the repos to mit hosted Github</t>
+        </is>
+      </c>
+      <c r="X128" s="13" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="37" t="inlineStr">
+        <is>
+          <t>Review the falut codes and connect to the error code excel</t>
+        </is>
+      </c>
+      <c r="X129" s="13" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="37" t="n"/>
+      <c r="X130" s="29" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="37" t="inlineStr">
+        <is>
+          <t>Reverse Enginginerg of the early criolife prototype</t>
+        </is>
+      </c>
+      <c r="X131" s="13" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="3" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="17" t="inlineStr">
+        <is>
+          <t>Intellectual Property</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
         <is>
           <t>Epic</t>
         </is>
       </c>
     </row>
-    <row r="77" hidden="1" s="26">
-      <c r="A77" s="5" t="inlineStr">
-        <is>
-          <t>Design</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" hidden="1" s="26">
-      <c r="A78" s="5" t="inlineStr">
-        <is>
-          <t>Order</t>
-        </is>
-      </c>
-    </row>
-    <row r="79" hidden="1" s="26">
-      <c r="A79" s="5" t="inlineStr">
-        <is>
-          <t>Integrate &amp; Test</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="5" t="inlineStr">
-        <is>
-          <t>Revise</t>
-        </is>
-      </c>
-    </row>
-    <row r="81" hidden="1" s="26">
-      <c r="A81" s="5" t="n"/>
-    </row>
-    <row r="82" hidden="1" s="26">
-      <c r="A82" s="17" t="inlineStr">
-        <is>
-          <t>Battery System</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" hidden="1" s="26">
-      <c r="A83" s="5" t="inlineStr">
-        <is>
-          <t>Integrate the Battery</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" hidden="1" s="26">
-      <c r="A84" s="5" t="inlineStr">
-        <is>
-          <t>Implement UI and Error cases</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" hidden="1" s="26">
-      <c r="A85" s="5" t="inlineStr">
-        <is>
-          <t>Test</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="5" t="inlineStr">
-        <is>
-          <t>Simulate 30min operation</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" hidden="1" s="26">
-      <c r="A87" s="25" t="inlineStr">
-        <is>
-          <t>Test whether USB-C input is an option</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Current Sprint</t>
-        </is>
-      </c>
-      <c r="X87" s="31" t="n"/>
-    </row>
-    <row r="88" hidden="1" s="26">
-      <c r="A88" s="2" t="n"/>
-    </row>
-    <row r="89" hidden="1" s="26">
-      <c r="A89" s="17" t="inlineStr">
-        <is>
-          <t>Sage Test Setup</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="5" t="inlineStr">
-        <is>
-          <t>Design and order</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" hidden="1" s="26">
-      <c r="A91" s="5" t="inlineStr">
-        <is>
-          <t>Build</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" hidden="1" s="26"/>
-    <row r="93" hidden="1" s="26">
-      <c r="A93" s="17" t="inlineStr">
-        <is>
-          <t>Prep for Animal Study</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" hidden="1" s="26">
-      <c r="A94" s="5" t="inlineStr">
-        <is>
-          <t>Study previous experiments</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="5" t="inlineStr">
-        <is>
-          <t>Desing the Study protocol - especially probe placement</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" hidden="1" s="26">
-      <c r="A96" s="5" t="inlineStr">
-        <is>
-          <t>Freeze the software/hardware version and conduct final verification</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" hidden="1" s="26">
-      <c r="A97" s="3" t="n"/>
-    </row>
-    <row r="98" hidden="1" s="26">
-      <c r="A98" s="17" t="inlineStr">
-        <is>
-          <t>Intellectual Property</t>
-        </is>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Epic</t>
-        </is>
-      </c>
-    </row>
-    <row r="99" hidden="1" s="26">
-      <c r="A99" s="5" t="inlineStr">
+    <row r="134">
+      <c r="A134" s="38" t="inlineStr">
         <is>
           <t>Internal Innovation Review - ID potential new IP</t>
         </is>
       </c>
     </row>
-    <row r="100" hidden="1" s="26">
-      <c r="A100" s="5" t="inlineStr">
+    <row r="135">
+      <c r="A135" s="38" t="inlineStr">
         <is>
           <t>Review pertinent prior art</t>
         </is>
       </c>
     </row>
-    <row r="101" hidden="1" s="26">
-      <c r="A101" s="5" t="inlineStr">
+    <row r="136">
+      <c r="A136" s="38" t="inlineStr">
         <is>
           <t>Review prior art</t>
         </is>
       </c>
     </row>
-    <row r="102" hidden="1" s="26">
-      <c r="A102" s="5" t="inlineStr">
+    <row r="137">
+      <c r="A137" s="38" t="inlineStr">
         <is>
           <t>Submit IP disclosure</t>
         </is>
       </c>
     </row>
-    <row r="103" hidden="1" s="26">
-      <c r="A103" s="5" t="n"/>
-    </row>
-    <row r="104" hidden="1" s="26">
-      <c r="A104" s="6" t="inlineStr">
+    <row r="138">
+      <c r="A138" s="38" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="6" t="inlineStr">
         <is>
           <t>Documentation</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="5" t="inlineStr">
+    <row r="140">
+      <c r="A140" s="38" t="inlineStr">
         <is>
           <t>Build documentation package</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="5" t="inlineStr">
+    <row r="141">
+      <c r="A141" s="38" t="inlineStr">
         <is>
           <t>Identify next potential partners</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="5" t="inlineStr">
+    <row r="142">
+      <c r="A142" s="38" t="inlineStr">
         <is>
           <t>Conduct tranfer</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="B108" s="16" t="inlineStr">
+    <row r="143">
+      <c r="A143" s="38" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="17" t="inlineStr">
+        <is>
+          <t>Cadaver Test</t>
+        </is>
+      </c>
+      <c r="B144" s="16" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="1" t="inlineStr">
+      <c r="AB144" s="13" t="n"/>
+      <c r="AC144" s="13" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="38" t="inlineStr">
+        <is>
+          <t>Create protokoll</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="38" t="inlineStr">
+        <is>
+          <t>conducts</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="38" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="17" t="inlineStr">
+        <is>
+          <t>Testing</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="38" t="inlineStr">
+        <is>
+          <t>Sous vide</t>
+        </is>
+      </c>
+      <c r="V149" s="13" t="n"/>
+      <c r="W149" s="30" t="n"/>
+      <c r="X149" s="13" t="n"/>
+      <c r="Y149" s="13" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="38" t="inlineStr">
+        <is>
+          <t>bain marie test</t>
+        </is>
+      </c>
+      <c r="Y150" s="13" t="n"/>
+      <c r="Z150" s="13" t="n"/>
+      <c r="AA150" s="13" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="38" t="n"/>
+      <c r="Y151" s="13" t="n"/>
+      <c r="Z151" s="13" t="n"/>
+      <c r="AA151" s="13" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="1" t="inlineStr">
         <is>
           <t>Non GLP Animal Study</t>
         </is>
       </c>
-      <c r="B109" s="16" t="inlineStr">
+      <c r="B152" s="16" t="inlineStr">
         <is>
           <t>Milestone</t>
         </is>
       </c>
-      <c r="AI109" s="30" t="n"/>
-    </row>
-    <row r="110">
-      <c r="A110" s="1" t="inlineStr">
+      <c r="AI152" s="26" t="n"/>
+    </row>
+    <row r="153" s="36">
+      <c r="A153" s="1" t="inlineStr">
         <is>
           <t>GLP Animla Study</t>
         </is>
       </c>
-      <c r="AO110" s="30" t="n"/>
+      <c r="AO153" s="26" t="n"/>
+    </row>
+    <row r="154" s="36">
+      <c r="A154" s="39" t="inlineStr">
+        <is>
+          <t>Electromagnetic compatibility testing</t>
+        </is>
+      </c>
+      <c r="AD154" s="27" t="n"/>
+      <c r="AE154" s="27" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A5:AW110">
-    <filterColumn colId="1" hiddenButton="0" showButton="1">
-      <filters>
-        <filter val="Current Sprint"/>
-        <filter val="Epic"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A5:AW154"/>
   <mergeCells count="9">
     <mergeCell ref="AD2:AI2"/>
     <mergeCell ref="AP2:AV2"/>
@@ -1811,13 +2149,18 @@
     <mergeCell ref="AD1:AW1"/>
     <mergeCell ref="P2:V2"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:AX102">
+  <conditionalFormatting sqref="A5:AX45 A46 A50:AX74 A75:Y75 A76:AX82 A83:X84 A85:AX137 Z83:AX84 AA75:AX75">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$C5="Yes"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="Y83">
+    <cfRule type="expression" priority="3" dxfId="0">
+      <formula>$C84="Yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="B6:B110" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid sprint status" error="Choose a value from the sprint-status list." type="list">
+    <dataValidation sqref="B6:B154" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid sprint status" error="Choose a value from the sprint-status list." type="list">
       <formula1>"Done,Last Sprint,Current Sprint,Next Sprint,Epic"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>